<commit_message>
feat: alle 30 Artikel mit CHECK24- & Tarifcheck-Affiliate-Links (PID 80968 / partner_id 47086); neuer Artikel Private Unfallversicherung; Verlinkungsplan-Excel mit Affiliate-Sheet aktualisiert
</commit_message>
<xml_diff>
--- a/Pinterest-Blog-Verlinkungsplan.xlsx
+++ b/Pinterest-Blog-Verlinkungsplan.xlsx
@@ -9,10 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verlinkungsplan" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blog-Artikel-URLs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Affiliate-Links" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Verlinkungsplan'!$A$1:$H$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Blog-Artikel-URLs'!$A$1:$D$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Affiliate-Links'!$A$1:$D$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -38,7 +41,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +61,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF3D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -87,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -106,6 +119,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2879,11 +2894,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="95" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2897,6 +2914,16 @@
           <t>URL</t>
         </is>
       </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Affiliate-Anbieter</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Affiliate-Link</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
@@ -2909,6 +2936,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
         </is>
       </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -2921,6 +2958,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
         </is>
       </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -2933,6 +2980,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
         </is>
       </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=dsl-anbieterwechsel&amp;cat=4</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -2945,6 +3002,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/dsl-internet-flat-guenstig-sichern/</t>
         </is>
       </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=dsl-anbieterwechsel&amp;cat=4</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -2957,6 +3024,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/e-auto-laden-stromkosten-senken/</t>
         </is>
       </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=stromanbieter-wechseln&amp;cat=1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -2969,6 +3046,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
         </is>
       </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -2981,6 +3068,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/gastarife-vergleichen-vor-dem-herbst/</t>
         </is>
       </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=gasanbieter-wechseln&amp;cat=3</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -2993,6 +3090,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/guenstige-fluege-spaetsommer-finden/</t>
         </is>
       </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=flugvergleich</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -3005,6 +3112,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/handytarife-vergleichen-guenstigster-tarif/</t>
         </is>
       </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=handytarife</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -3017,6 +3134,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/hausratversicherung-wer-braucht-leistung/</t>
         </is>
       </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Tarifcheck</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=hausratversicherung</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -3029,6 +3156,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
         </is>
       </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=gasanbieter-wechseln&amp;cat=3</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -3041,6 +3178,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/kfz-versicherung-wechseln/</t>
         </is>
       </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kfz-versicherung</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -3053,6 +3200,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/kostenloses-girokonto-finden/</t>
         </is>
       </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=c24bank&amp;cat=14</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -3065,6 +3222,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/kreditkarte-ohne-jahresgebuehr/</t>
         </is>
       </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kreditkarte</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -3077,6 +3244,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/last-minute-urlaubsangebote-sichern/</t>
         </is>
       </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=pauschalreisen-vergleich&amp;cat=9</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -3089,6 +3266,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/mietwagen-buchen-so-sparst-du/</t>
         </is>
       </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=mietwagen-preisvergleich&amp;cat=10</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -3101,6 +3288,16 @@
           <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
         </is>
       </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=mietwagen-preisvergleich&amp;cat=10</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -3113,140 +3310,283 @@
           <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
         </is>
       </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=c24bank&amp;cat=14</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Privathaftpflicht: Warum sie Pflicht ist und was sie kostet</t>
+          <t>Private Unfallversicherung: Für wen sie sich wirklich lohnt</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/privathaftpflicht-warum-pflicht-kosten/</t>
+          <t>https://DEINE-DOMAIN.DE/posts/private-unfallversicherung-fuer-wen-sie-sich-wirklich-lohnt/</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Tarifcheck</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=unfallversicherung</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Günstigen Ratenkredit mit Bestzins sichern: So vergleichst du richtig</t>
+          <t>Privathaftpflicht: Warum sie Pflicht ist und was sie kostet</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/ratenkredit-bestszins-vergleichen/</t>
+          <t>https://DEINE-DOMAIN.DE/posts/privathaftpflicht-warum-pflicht-kosten/</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Tarifcheck</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=haftpflichtversicherung</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Reisekrankenversicherung: Wann sie sich wirklich lohnt</t>
+          <t>Günstigen Ratenkredit mit Bestzins sichern: So vergleichst du richtig</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/reisekrankenversicherung-wann-lohnt/</t>
+          <t>https://DEINE-DOMAIN.DE/posts/ratenkredit-bestszins-vergleichen/</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kreditvergleich</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Strom sparen im Haushalt: 20 Tipps für die nächste Rechnung</t>
+          <t>Reisekrankenversicherung: Wann sie sich wirklich lohnt</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/strom-sparen-haushalt-20-tipps/</t>
+          <t>https://DEINE-DOMAIN.DE/posts/reisekrankenversicherung-wann-lohnt/</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Tarifcheck</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=reisekrankenversicherung</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Stromanbieter wechseln: So sparst du 2026 bis zu 300 € im Jahr</t>
+          <t>Strom sparen im Haushalt: 20 Tipps für die nächste Rechnung</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromanbieter-wechseln-2026/</t>
+          <t>https://DEINE-DOMAIN.DE/posts/strom-sparen-haushalt-20-tipps/</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=stromanbieter-wechseln&amp;cat=1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Stromfresser im Haushalt entlarven: Diese 3 Geräte treiben deine Stromrechnung hoch</t>
+          <t>Stromanbieter wechseln: So sparst du 2026 bis zu 300 € im Jahr</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+          <t>https://DEINE-DOMAIN.DE/posts/stromanbieter-wechseln-2026/</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=stromanbieter-wechseln&amp;cat=1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Tagesgeld und Zinsen: So parkst du dein Geld sicher</t>
+          <t>Stromfresser im Haushalt entlarven: Diese 3 Geräte treiben deine Stromrechnung hoch</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/tagesgeld-zinsen-sicher-anlegen/</t>
+          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=stromanbieter-wechseln&amp;cat=1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Urlaubskasse clever aufbessern: 7 erprobte Spartipps für den Sommerurlaub</t>
+          <t>Tagesgeld und Zinsen: So parkst du dein Geld sicher</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+          <t>https://DEINE-DOMAIN.DE/posts/tagesgeld-zinsen-sicher-anlegen/</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=tagesgeldvergleich</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Wärmepumpe vs. Gasheizung: Was lohnt sich 2026?</t>
+          <t>Urlaubskasse clever aufbessern: 7 erprobte Spartipps für den Sommerurlaub</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/waermepumpe-vs-gasheizung-2026/</t>
+          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=pauschalreisen-vergleich&amp;cat=9</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>WLAN-Verstärker vs. Mesh-WLAN: So bekommst du überall schnelles Internet</t>
+          <t>Wärmepumpe vs. Gasheizung: Was lohnt sich 2026?</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+          <t>https://DEINE-DOMAIN.DE/posts/waermepumpe-vs-gasheizung-2026/</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=stromanbieter-wechseln&amp;cat=1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
+          <t>WLAN-Verstärker vs. Mesh-WLAN: So bekommst du überall schnelles Internet</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=dsl-anbieterwechsel&amp;cat=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
           <t>Zahnzusatzversicherung: Lohnt sich der Abschluss?</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>https://DEINE-DOMAIN.DE/posts/zahnzusatzversicherung-lohnt-sich/</t>
         </is>
       </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Tarifcheck</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=zahnzusatzversicherung</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3257,16 +3597,455 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="110" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
-        <is>
-          <t>Pinterest-Verknüpfung – So stellst du sie ein</t>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Kategorie</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Anbieter</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=stromanbieter-wechseln&amp;cat=1</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>PDF bestätigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=gasanbieter-wechseln&amp;cat=3</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>PDF bestätigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>DSL/Internet</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=dsl-anbieterwechsel&amp;cat=4</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>PDF bestätigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Mietwagen</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=mietwagen-preisvergleich&amp;cat=10</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>PDF bestätigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Pauschalreisen</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=pauschalreisen-vergleich&amp;cat=9</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>PDF bestätigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Girokonto (C24)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=c24bank&amp;cat=14</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>PDF bestätigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Allgemein</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>PDF bestätigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Unfallversicherung</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Tarifcheck</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=unfallversicherung</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>PDF bestätigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Kredit</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kreditvergleich</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Muster getestet</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Kfz-Versicherung</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kfz-versicherung</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Muster getestet</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Flüge</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=flugvergleich</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Muster getestet</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Handytarife</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=handytarife</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Muster getestet</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Kreditkarte</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kreditkarte</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Muster getestet</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Tagesgeld</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=tagesgeldvergleich</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Muster getestet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Haftpflicht</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Tarifcheck</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=haftpflichtversicherung</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Muster getestet</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Hausrat</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Tarifcheck</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=hausratversicherung</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Muster getestet</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Zahnzusatz</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Tarifcheck</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=zahnzusatzversicherung</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Muster getestet</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Reisekrankenversicherung</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Tarifcheck</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=reisekrankenversicherung</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Muster getestet</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D19"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Pinterest-Verknüpfung &amp; Affiliate-Links – Anleitung</t>
         </is>
       </c>
     </row>
@@ -3283,7 +4062,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   DEINE-DOMAIN.DE durch deine echte Domain ersetzen (z. B. www.franksfinanzcheck.de).</t>
+          <t xml:space="preserve">   DEINE-DOMAIN.DE durch deine echte Domain ersetzen.</t>
         </is>
       </c>
     </row>
@@ -3303,69 +4082,69 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3. In Pinterest: Für jeden Pin die 'Destination-URL' auf die neue Blog-URL ändern.</t>
+          <t>3. In Pinterest: Für jeden Pin die 'Destination-URL' auf die neue Blog-URL ändern</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Das geht einzeln im Pin-Editor – oder schneller über den Bulk-Editor</t>
+          <t xml:space="preserve">   (einzeln im Pin-Editor oder über den Bulk-Editor).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   (Pinterest Business Hub → Pin-Editor → mehrere Pins markieren → URL ändern).</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>4. AFFILIATE-LINKS: Alle 30 Artikel verlinken bereits mit deiner PID 80968</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>4. Tipp: Die Educational-Pins (EP) führen Besucher jetzt auf deinen Blog</t>
+          <t xml:space="preserve">   (CHECK24) bzw. partner_id 47086 (Tarifcheck). Siehe Sheet 'Affiliate-Links'.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   statt auf dein Pinterest-Profil – so bleibt der Traffic auf deiner eigenen Seite</t>
+          <t xml:space="preserve">   - CHECK24-Kategorien: Strom, Gas, DSL, Mietwagen, Reisen, Girokonto, Kredit,</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   und stärkt dein SEO-Ranking (interne Verlinkung + Backlinks von Pinterest).</t>
+          <t xml:space="preserve">     Kfz, Flüge, Handytarife, Kreditkarte, Tagesgeld + allgemein</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Tarifcheck-Kategorien: Unfall, Haftpflicht, Hausrat, Zahnzusatz, Reisekranken</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>5. Die Transactional-Pins (TP) verlinken auf den passenden Blog-Artikel,</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   der wiederum deinen persönlichen CHECK24-Link enthält.</t>
+          <t>5. Neue Artikel: python3 scripts/set_check24_links.py --topics ausführen,</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Wichtig: Vorher scripts/set_check24_links.py --id DEINE_ID --topics ausführen!</t>
+          <t xml:space="preserve">   dann sind auch neue Bot-Artikel automatisch mit deinen Links versehen.</t>
         </is>
       </c>
     </row>
@@ -3375,14 +4154,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>6. Nach dem Umstellen: Pins neu pinnen bzw. den Pin aktualisieren,</t>
+          <t>6. Hinweis: Die mit 'Muster getestet' markierten Links wurden per HTTP-Test</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   damit Pinterest die neue URL crawlt.</t>
+          <t xml:space="preserve">   verifiziert (301-Weiterleitung mit PID). Bitte zur Sicherheit im Partner-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Dashboard gegenprüfen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: Verlinkungsplan-Excel überarbeitet – TP-Pins verlinken direkt auf Affiliate-Links, EP-Pins auf Blog-Artikel; neue Spalten Strategie/Anbieter; Anleitung aktualisiert
</commit_message>
<xml_diff>
--- a/Pinterest-Blog-Verlinkungsplan.xlsx
+++ b/Pinterest-Blog-Verlinkungsplan.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Verlinkungsplan'!$A$1:$H$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Verlinkungsplan'!$A$1:$J$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Blog-Artikel-URLs'!$A$1:$D$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Affiliate-Links'!$A$1:$D$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Affiliate-Links'!$A$1:$D$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -38,7 +38,7 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="13"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="7">
@@ -103,7 +103,7 @@
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -487,17 +487,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:J63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -533,12 +535,22 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Blog-Artikel</t>
+          <t>Ziel-Strategie</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Neue Destination-URL</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (bei EP)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Affiliate-Anbieter</t>
         </is>
       </c>
     </row>
@@ -569,14 +581,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>5 einfache Frugalismus-Tricks für den Alltag: So sparst du 200 € im Monat</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -607,14 +629,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Die 50-30-20-Regel einfach erklärt: Die perfekte Formel für deine Finanzen</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -645,14 +677,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Stromfresser im Haushalt entlarven: Diese 3 Geräte treiben deine Stromrechnung hoch</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -683,14 +725,24 @@
           <t>https://www.check24.de/strom/</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Stromanbieter wechseln: So sparst du 2026 bis zu 300 € im Jahr</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromanbieter-wechseln-2026/</t>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Direkt auf Affiliate-Link</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=stromanbieter-wechseln&amp;cat=1</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>(Art. Stromanbieter wechseln: So sparst du 2026 bis zu 300 € im Jahr)</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
         </is>
       </c>
     </row>
@@ -717,14 +769,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>WLAN-Verstärker vs. Mesh-WLAN: So bekommst du überall schnelles Internet</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -755,14 +817,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Urlaubskasse clever aufbessern: 7 erprobte Spartipps für den Sommerurlaub</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -793,14 +865,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>7 Gewohnheiten für finanzielle Freiheit: Kleine Schritte, große Wirkung</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -831,14 +913,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Notgroschen aufbauen: Wie viel Geld reicht wirklich?</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -869,14 +961,24 @@
           <t>https://www.check24.de/gas/</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>Gastarife vergleichen vor dem Herbst: So senkst du deine Heizkosten</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/gastarife-vergleichen-vor-dem-herbst/</t>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Direkt auf Affiliate-Link</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=gasanbieter-wechseln&amp;cat=3</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>(Art. Gastarife vergleichen vor dem Herbst: So senkst du deine Heizkosten)</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
         </is>
       </c>
     </row>
@@ -907,14 +1009,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Heizperiode vorbereiten im Spätsommer: 3 Dinge, die du im August tun musst</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -945,14 +1057,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>DNS-Server ändern: Der kostenlose Boost für dein Internet</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -983,14 +1105,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Mietwagen-Fallen im Urlaub vermeiden: Worauf du bei Versicherung &amp; Kaution achten musst</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1021,14 +1153,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>5 einfache Frugalismus-Tricks für den Alltag: So sparst du 200 € im Monat</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1059,14 +1201,24 @@
           <t>https://www.check24.de/dsl/</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>DSL- und Internet-Flat günstig sichern: So findest du den besten Tarif</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dsl-internet-flat-guenstig-sichern/</t>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Direkt auf Affiliate-Link</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=dsl-anbieterwechsel&amp;cat=4</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>(Art. DSL- und Internet-Flat günstig sichern: So findest du den besten Tarif)</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
         </is>
       </c>
     </row>
@@ -1097,14 +1249,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>Die 50-30-20-Regel einfach erklärt: Die perfekte Formel für deine Finanzen</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1135,14 +1297,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>Stromfresser im Haushalt entlarven: Diese 3 Geräte treiben deine Stromrechnung hoch</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1169,14 +1341,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>WLAN-Verstärker vs. Mesh-WLAN: So bekommst du überall schnelles Internet</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1207,14 +1389,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>Urlaubskasse clever aufbessern: 7 erprobte Spartipps für den Sommerurlaub</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1245,14 +1437,24 @@
           <t>https://www.check24.de/girokonto/</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>Kostenloses Girokonto ohne Gebühren: So findest du das richtige</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/kostenloses-girokonto-finden/</t>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Direkt auf Affiliate-Link</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=c24bank&amp;cat=14</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>(Art. Kostenloses Girokonto ohne Gebühren: So findest du das richtige)</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
         </is>
       </c>
     </row>
@@ -1283,14 +1485,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>7 Gewohnheiten für finanzielle Freiheit: Kleine Schritte, große Wirkung</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1321,14 +1533,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>Notgroschen aufbauen: Wie viel Geld reicht wirklich?</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1359,14 +1581,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>Heizperiode vorbereiten im Spätsommer: 3 Dinge, die du im August tun musst</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1397,14 +1629,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>DNS-Server ändern: Der kostenlose Boost für dein Internet</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1435,14 +1677,24 @@
           <t>https://www.check24.de/kredit/</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>Günstigen Ratenkredit mit Bestzins sichern: So vergleichst du richtig</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/ratenkredit-bestszins-vergleichen/</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Direkt auf Affiliate-Link</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kreditvergleich</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>(Art. Günstigen Ratenkredit mit Bestzins sichern: So vergleichst du richtig)</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
         </is>
       </c>
     </row>
@@ -1469,14 +1721,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
         <is>
           <t>Mietwagen-Fallen im Urlaub vermeiden: Worauf du bei Versicherung &amp; Kaution achten musst</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1507,14 +1769,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>5 einfache Frugalismus-Tricks für den Alltag: So sparst du 200 € im Monat</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1545,14 +1817,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>Die 50-30-20-Regel einfach erklärt: Die perfekte Formel für deine Finanzen</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1583,14 +1865,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>Stromfresser im Haushalt entlarven: Diese 3 Geräte treiben deine Stromrechnung hoch</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1621,14 +1913,24 @@
           <t>https://www.check24.de/kfz-versicherung/</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
-        <is>
-          <t>Kfz-Versicherung wechseln: Wann sich der Wechsel wirklich lohnt</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/kfz-versicherung-wechseln/</t>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Direkt auf Affiliate-Link</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kfz-versicherung</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>(Art. Kfz-Versicherung wechseln: Wann sich der Wechsel wirklich lohnt)</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
         </is>
       </c>
     </row>
@@ -1659,14 +1961,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>WLAN-Verstärker vs. Mesh-WLAN: So bekommst du überall schnelles Internet</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1697,14 +2009,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
         <is>
           <t>Urlaubskasse clever aufbessern: 7 erprobte Spartipps für den Sommerurlaub</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1735,14 +2057,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
         <is>
           <t>7 Gewohnheiten für finanzielle Freiheit: Kleine Schritte, große Wirkung</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1773,14 +2105,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>Notgroschen aufbauen: Wie viel Geld reicht wirklich?</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1811,14 +2153,24 @@
           <t>https://www.check24.de/reisen/</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>Last-Minute Urlaubsangebote sichern: So buchst du den Traumurlaub günstig</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/last-minute-urlaubsangebote-sichern/</t>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Direkt auf Affiliate-Link</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=pauschalreisen-vergleich&amp;cat=9</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>(Art. Last-Minute Urlaubsangebote sichern: So buchst du den Traumurlaub günstig)</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
         </is>
       </c>
     </row>
@@ -1849,14 +2201,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
         <is>
           <t>Heizperiode vorbereiten im Spätsommer: 3 Dinge, die du im August tun musst</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1887,14 +2249,24 @@
           <t>https://www.pinterest.denrankstinanzcheck/</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
         <is>
           <t>DNS-Server ändern: Der kostenlose Boost für dein Internet</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1925,14 +2297,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
         <is>
           <t>Mietwagen-Fallen im Urlaub vermeiden: Worauf du bei Versicherung &amp; Kaution achten musst</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -1963,14 +2345,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
         <is>
           <t>5 einfache Frugalismus-Tricks für den Alltag: So sparst du 200 € im Monat</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2001,14 +2393,24 @@
           <t>https://www.check24.de/mietwagen/</t>
         </is>
       </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>Günstigen Mietwagen für den Urlaub buchen: So sparst du richtig</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-buchen-so-sparst-du/</t>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>Direkt auf Affiliate-Link</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=mietwagen-preisvergleich&amp;cat=10</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>(Art. Günstigen Mietwagen für den Urlaub buchen: So sparst du richtig)</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
         </is>
       </c>
     </row>
@@ -2039,14 +2441,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
         <is>
           <t>Die 50-30-20-Regel einfach erklärt: Die perfekte Formel für deine Finanzen</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2077,14 +2489,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G42" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
         <is>
           <t>Stromfresser im Haushalt entlarven: Diese 3 Geräte treiben deine Stromrechnung hoch</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2115,14 +2537,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
         <is>
           <t>WLAN-Verstärker vs. Mesh-WLAN: So bekommst du überall schnelles Internet</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2153,14 +2585,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G44" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
         <is>
           <t>Urlaubskasse clever aufbessern: 7 erprobte Spartipps für den Sommerurlaub</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2187,14 +2629,24 @@
           <t>https://www.check24.de/fluege/</t>
         </is>
       </c>
-      <c r="G45" s="5" t="inlineStr">
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/guenstige-fluege-spaetsommer-finden/</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
         <is>
           <t>Günstige Flüge für den Spätsommer finden: 7 Tricks, die wirklich funktionieren</t>
         </is>
       </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/guenstige-fluege-spaetsommer-finden/</t>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2225,14 +2677,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G46" s="3" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
         <is>
           <t>7 Gewohnheiten für finanzielle Freiheit: Kleine Schritte, große Wirkung</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2263,14 +2725,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
         <is>
           <t>Notgroschen aufbauen: Wie viel Geld reicht wirklich?</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2301,14 +2773,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G48" s="3" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
         <is>
           <t>Heizperiode vorbereiten im Spätsommer: 3 Dinge, die du im August tun musst</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2339,14 +2821,24 @@
           <t>https://www.pinterest.denranksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
         <is>
           <t>DNS-Server ändern: Der kostenlose Boost für dein Internet</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2377,14 +2869,24 @@
           <t>https://www.check24.de/gas/</t>
         </is>
       </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>Gastarife vergleichen vor dem Herbst: So senkst du deine Heizkosten</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/gastarife-vergleichen-vor-dem-herbst/</t>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>Direkt auf Affiliate-Link</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=gasanbieter-wechseln&amp;cat=3</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>(Art. Gastarife vergleichen vor dem Herbst: So senkst du deine Heizkosten)</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
         </is>
       </c>
     </row>
@@ -2415,14 +2917,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
         <is>
           <t>Mietwagen-Fallen im Urlaub vermeiden: Worauf du bei Versicherung &amp; Kaution achten musst</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2453,14 +2965,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G52" s="3" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
         <is>
           <t>5 einfache Frugalismus-Tricks für den Alltag: So sparst du 200 € im Monat</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2491,14 +3013,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
         <is>
           <t>Die 50-30-20-Regel einfach erklärt: Die perfekte Formel für deine Finanzen</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2529,14 +3061,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G54" s="3" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
         <is>
           <t>Stromfresser im Haushalt entlarven: Diese 3 Geräte treiben deine Stromrechnung hoch</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2567,14 +3109,24 @@
           <t>https://www.check24.de/dsl/</t>
         </is>
       </c>
-      <c r="G55" s="5" t="inlineStr">
-        <is>
-          <t>DSL- und Internet-Flat günstig sichern: So findest du den besten Tarif</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dsl-internet-flat-guenstig-sichern/</t>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>Direkt auf Affiliate-Link</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=dsl-anbieterwechsel&amp;cat=4</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>(Art. DSL- und Internet-Flat günstig sichern: So findest du den besten Tarif)</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
         </is>
       </c>
     </row>
@@ -2605,14 +3157,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G56" s="3" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
         <is>
           <t>WLAN-Verstärker vs. Mesh-WLAN: So bekommst du überall schnelles Internet</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2643,14 +3205,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
         <is>
           <t>Urlaubskasse clever aufbessern: 7 erprobte Spartipps für den Sommerurlaub</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2681,14 +3253,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G58" s="3" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
         <is>
           <t>7 Gewohnheiten für finanzielle Freiheit: Kleine Schritte, große Wirkung</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2719,14 +3301,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G59" s="3" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
         <is>
           <t>Notgroschen aufbauen: Wie viel Geld reicht wirklich?</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2757,14 +3349,24 @@
           <t>https://www.check24.de/mietwagen/</t>
         </is>
       </c>
-      <c r="G60" s="5" t="inlineStr">
-        <is>
-          <t>Günstigen Mietwagen für den Urlaub buchen: So sparst du richtig</t>
-        </is>
-      </c>
-      <c r="H60" s="4" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-buchen-so-sparst-du/</t>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>Direkt auf Affiliate-Link</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=mietwagen-preisvergleich&amp;cat=10</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>(Art. Günstigen Mietwagen für den Urlaub buchen: So sparst du richtig)</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
         </is>
       </c>
     </row>
@@ -2795,14 +3397,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G61" s="3" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
         <is>
           <t>Heizperiode vorbereiten im Spätsommer: 3 Dinge, die du im August tun musst</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2833,14 +3445,24 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G62" s="3" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
         <is>
           <t>DNS-Server ändern: Der kostenlose Boost für dein Internet</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
@@ -2871,19 +3493,29 @@
           <t>https://www.pinterest.de/franksfinanzcheck/</t>
         </is>
       </c>
-      <c r="G63" s="3" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Blog-Artikel (enthält Affiliate-Link)</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
         <is>
           <t>Mietwagen-Fallen im Urlaub vermeiden: Worauf du bei Versicherung &amp; Kaution achten musst</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr">
-        <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>CHECK24/Tarifcheck im Artikel</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H63"/>
+  <autoFilter ref="A1:J63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3597,7 +4229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3631,7 +4263,7 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Strom</t>
+          <t>strom</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -3653,7 +4285,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Gas</t>
+          <t>gas</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -3675,7 +4307,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>DSL/Internet</t>
+          <t>dsl</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -3697,7 +4329,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Mietwagen</t>
+          <t>mietwagen</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -3719,7 +4351,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Pauschalreisen</t>
+          <t>reisen</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -3741,7 +4373,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Girokonto (C24)</t>
+          <t>girokonto</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -3763,7 +4395,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Allgemein</t>
+          <t>kredit</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -3773,41 +4405,41 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18</t>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kreditvergleich</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>PDF bestätigt</t>
+          <t>Muster getestet</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Unfallversicherung</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Tarifcheck</t>
+          <t>kfz-versicherung</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>CHECK24</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=unfallversicherung</t>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kfz-versicherung</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>PDF bestätigt</t>
+          <t>Muster getestet</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Kredit</t>
+          <t>fluege</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -3817,7 +4449,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kreditvergleich</t>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=flugvergleich</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -3829,7 +4461,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Kfz-Versicherung</t>
+          <t>handytarife</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -3839,7 +4471,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kfz-versicherung</t>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=handytarife</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -3851,7 +4483,7 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Flüge</t>
+          <t>kreditkarte</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -3861,7 +4493,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=flugvergleich</t>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kreditkarte</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -3873,7 +4505,7 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Handytarife</t>
+          <t>tagesgeld</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -3883,7 +4515,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=handytarife</t>
+          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=tagesgeldvergleich</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -3895,39 +4527,39 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Kreditkarte</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>CHECK24</t>
+          <t>unfallversicherung</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Tarifcheck</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=kreditkarte</t>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=unfallversicherung</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Muster getestet</t>
+          <t>PDF bestätigt</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Tagesgeld</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>CHECK24</t>
+          <t>haftpflicht</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Tarifcheck</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>https://a.check24.net/misc/click.php?pid=80968&amp;aid=18&amp;deep=tagesgeldvergleich</t>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=haftpflichtversicherung</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -3939,7 +4571,7 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Haftpflicht</t>
+          <t>hausrat</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
@@ -3949,7 +4581,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=haftpflichtversicherung</t>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=hausratversicherung</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -3961,7 +4593,7 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Hausrat</t>
+          <t>zahnzusatzversicherung</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
@@ -3971,7 +4603,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=hausratversicherung</t>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=zahnzusatzversicherung</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -3983,7 +4615,7 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Zahnzusatz</t>
+          <t>reisekrankenversicherung</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
@@ -3993,7 +4625,7 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=zahnzusatzversicherung</t>
+          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=reisekrankenversicherung</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -4002,30 +4634,8 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Reisekrankenversicherung</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>Tarifcheck</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>https://a.partner-versicherung.de/click.php?partner_id=47086&amp;ad_id=15&amp;deep=reisekrankenversicherung</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>Muster getestet</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D19"/>
+  <autoFilter ref="A1:D18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4036,16 +4646,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="115" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>Pinterest-Verknüpfung &amp; Affiliate-Links – Anleitung</t>
+          <t>Pinterest-Verknüpfung &amp; Affiliate-Links – Anleitung (aktualisiert)</t>
         </is>
       </c>
     </row>
@@ -4053,122 +4663,165 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1. Domain ersetzen: In dieser Datei und in hugo.toml (baseURL) den Platzhalter</t>
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>STRATEGIE:</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   DEINE-DOMAIN.DE durch deine echte Domain ersetzen.</t>
+          <t>- Educational-Pins (EP, grün): → Blog-Artikel (URL unten). Der Artikel</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  enthält den passenden Affiliate-Link – so bleibt der Traffic auf deiner Seite.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2. Blog veröffentlichen (siehe README): GitHub Pages / Cloudflare Pages / Netlify.</t>
+          <t>- Transactional-Pins (TP, gelb): → DIREKT auf deinen Affiliate-Link</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (a.check24.net / a.partner-versicherung.de). Diese Pins sind Werbung</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3. In Pinterest: Für jeden Pin die 'Destination-URL' auf die neue Blog-URL ändern</t>
+          <t xml:space="preserve">  (#Anzeige) und sollen direkt zum Abschluss führen.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   (einzeln im Pin-Editor oder über den Bulk-Editor).</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>SCHRITTE:</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>4. AFFILIATE-LINKS: Alle 30 Artikel verlinken bereits mit deiner PID 80968</t>
+          <t>1. Domain ersetzen: In der Excel-Spalte 'Neue Destination-URL' bei EP-Pins</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (CHECK24) bzw. partner_id 47086 (Tarifcheck). Siehe Sheet 'Affiliate-Links'.</t>
+          <t xml:space="preserve">   DEINE-DOMAIN.DE durch deine echte Domain ersetzen (hugo.toml baseURL).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - CHECK24-Kategorien: Strom, Gas, DSL, Mietwagen, Reisen, Girokonto, Kredit,</t>
+          <t>2. Blog veröffentlichen (siehe README).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Kfz, Flüge, Handytarife, Kreditkarte, Tagesgeld + allgemein</t>
+          <t>3. In Pinterest: Pin-Editor → Destination-URL eintragen:</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Tarifcheck-Kategorien: Unfall, Haftpflicht, Hausrat, Zahnzusatz, Reisekranken</t>
+          <t xml:space="preserve">   - EP-Pins: Blog-Artikel-URL</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - TP-Pins: Affiliate-Link (Spalte 'Neue Destination-URL')</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>5. Neue Artikel: python3 scripts/set_check24_links.py --topics ausführen,</t>
+          <t>4. Bulk-Editor nutzen, um mehrere Pins auf einmal zu ändern.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   dann sind auch neue Bot-Artikel automatisch mit deinen Links versehen.</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>AFFILIATE-LINKS:</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>6. Hinweis: Die mit 'Muster getestet' markierten Links wurden per HTTP-Test</t>
+          <t>- CHECK24 (PID 80968): Strom, Gas, DSL, Mietwagen, Reisen, Girokonto,</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   verifiziert (301-Weiterleitung mit PID). Bitte zur Sicherheit im Partner-</t>
+          <t xml:space="preserve">  Kredit, Kfz, Flüge, Handytarife, Kreditkarte, Tagesgeld</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Dashboard gegenprüfen.</t>
+          <t>- Tarifcheck (partner_id 47086): Unfall, Haftpflicht, Hausrat, Zahnzusatz,</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Reisekrankenversicherung</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>- 'Muster getestet' = per HTTP verifiziert, bitte im Dashboard gegenprüfen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>NEUE ARTIKEL: python3 scripts/set_check24_links.py --topics ausführen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>dann haben auch neue Bot-Artikel automatisch deine Affiliate-Links.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
config: baseURL auf franksfinanzcheck.de gesetzt; Excel-Verlinkungsplan auf echte Domain umgestellt
</commit_message>
<xml_diff>
--- a/Pinterest-Blog-Verlinkungsplan.xlsx
+++ b/Pinterest-Blog-Verlinkungsplan.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+          <t>https://franksfinanzcheck.de/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+          <t>https://franksfinanzcheck.de/posts/50-30-20-regel-einfach-erklaert/</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+          <t>https://franksfinanzcheck.de/posts/stromfresser-im-haushalt-entlarven/</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+          <t>https://franksfinanzcheck.de/posts/wlan-verstaerker-vs-mesh-wlan/</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+          <t>https://franksfinanzcheck.de/posts/urlaubskasse-aufbessern-spartipps/</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+          <t>https://franksfinanzcheck.de/posts/7-gewohnheiten-finanzielle-freiheit/</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+          <t>https://franksfinanzcheck.de/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+          <t>https://franksfinanzcheck.de/posts/heizperiode-vorbereiten-spaetsommer/</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+          <t>https://franksfinanzcheck.de/posts/dns-server-aendern-schnelleres-internet/</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+          <t>https://franksfinanzcheck.de/posts/mietwagen-fallen-vermeiden/</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+          <t>https://franksfinanzcheck.de/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+          <t>https://franksfinanzcheck.de/posts/50-30-20-regel-einfach-erklaert/</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+          <t>https://franksfinanzcheck.de/posts/stromfresser-im-haushalt-entlarven/</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+          <t>https://franksfinanzcheck.de/posts/wlan-verstaerker-vs-mesh-wlan/</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+          <t>https://franksfinanzcheck.de/posts/urlaubskasse-aufbessern-spartipps/</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+          <t>https://franksfinanzcheck.de/posts/7-gewohnheiten-finanzielle-freiheit/</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+          <t>https://franksfinanzcheck.de/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+          <t>https://franksfinanzcheck.de/posts/heizperiode-vorbereiten-spaetsommer/</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+          <t>https://franksfinanzcheck.de/posts/dns-server-aendern-schnelleres-internet/</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+          <t>https://franksfinanzcheck.de/posts/mietwagen-fallen-vermeiden/</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+          <t>https://franksfinanzcheck.de/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+          <t>https://franksfinanzcheck.de/posts/50-30-20-regel-einfach-erklaert/</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+          <t>https://franksfinanzcheck.de/posts/stromfresser-im-haushalt-entlarven/</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+          <t>https://franksfinanzcheck.de/posts/wlan-verstaerker-vs-mesh-wlan/</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+          <t>https://franksfinanzcheck.de/posts/urlaubskasse-aufbessern-spartipps/</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+          <t>https://franksfinanzcheck.de/posts/7-gewohnheiten-finanzielle-freiheit/</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+          <t>https://franksfinanzcheck.de/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+          <t>https://franksfinanzcheck.de/posts/heizperiode-vorbereiten-spaetsommer/</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+          <t>https://franksfinanzcheck.de/posts/dns-server-aendern-schnelleres-internet/</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+          <t>https://franksfinanzcheck.de/posts/mietwagen-fallen-vermeiden/</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+          <t>https://franksfinanzcheck.de/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+          <t>https://franksfinanzcheck.de/posts/50-30-20-regel-einfach-erklaert/</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+          <t>https://franksfinanzcheck.de/posts/stromfresser-im-haushalt-entlarven/</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+          <t>https://franksfinanzcheck.de/posts/wlan-verstaerker-vs-mesh-wlan/</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+          <t>https://franksfinanzcheck.de/posts/urlaubskasse-aufbessern-spartipps/</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/guenstige-fluege-spaetsommer-finden/</t>
+          <t>https://franksfinanzcheck.de/posts/guenstige-fluege-spaetsommer-finden/</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+          <t>https://franksfinanzcheck.de/posts/7-gewohnheiten-finanzielle-freiheit/</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+          <t>https://franksfinanzcheck.de/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+          <t>https://franksfinanzcheck.de/posts/heizperiode-vorbereiten-spaetsommer/</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
@@ -2828,7 +2828,7 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+          <t>https://franksfinanzcheck.de/posts/dns-server-aendern-schnelleres-internet/</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+          <t>https://franksfinanzcheck.de/posts/mietwagen-fallen-vermeiden/</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+          <t>https://franksfinanzcheck.de/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+          <t>https://franksfinanzcheck.de/posts/50-30-20-regel-einfach-erklaert/</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+          <t>https://franksfinanzcheck.de/posts/stromfresser-im-haushalt-entlarven/</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+          <t>https://franksfinanzcheck.de/posts/wlan-verstaerker-vs-mesh-wlan/</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+          <t>https://franksfinanzcheck.de/posts/urlaubskasse-aufbessern-spartipps/</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3260,7 +3260,7 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+          <t>https://franksfinanzcheck.de/posts/7-gewohnheiten-finanzielle-freiheit/</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
@@ -3308,7 +3308,7 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+          <t>https://franksfinanzcheck.de/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
@@ -3404,7 +3404,7 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+          <t>https://franksfinanzcheck.de/posts/heizperiode-vorbereiten-spaetsommer/</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
@@ -3452,7 +3452,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+          <t>https://franksfinanzcheck.de/posts/dns-server-aendern-schnelleres-internet/</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
@@ -3500,7 +3500,7 @@
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+          <t>https://franksfinanzcheck.de/posts/mietwagen-fallen-vermeiden/</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/50-30-20-regel-einfach-erklaert/</t>
+          <t>https://franksfinanzcheck.de/posts/50-30-20-regel-einfach-erklaert/</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/7-gewohnheiten-finanzielle-freiheit/</t>
+          <t>https://franksfinanzcheck.de/posts/7-gewohnheiten-finanzielle-freiheit/</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dns-server-aendern-schnelleres-internet/</t>
+          <t>https://franksfinanzcheck.de/posts/dns-server-aendern-schnelleres-internet/</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -3631,7 +3631,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/dsl-internet-flat-guenstig-sichern/</t>
+          <t>https://franksfinanzcheck.de/posts/dsl-internet-flat-guenstig-sichern/</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/e-auto-laden-stromkosten-senken/</t>
+          <t>https://franksfinanzcheck.de/posts/e-auto-laden-stromkosten-senken/</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
+          <t>https://franksfinanzcheck.de/posts/frugalismus-tricks-alltag-200-euro-sparen/</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/gastarife-vergleichen-vor-dem-herbst/</t>
+          <t>https://franksfinanzcheck.de/posts/gastarife-vergleichen-vor-dem-herbst/</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -3719,7 +3719,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/guenstige-fluege-spaetsommer-finden/</t>
+          <t>https://franksfinanzcheck.de/posts/guenstige-fluege-spaetsommer-finden/</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/handytarife-vergleichen-guenstigster-tarif/</t>
+          <t>https://franksfinanzcheck.de/posts/handytarife-vergleichen-guenstigster-tarif/</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/hausratversicherung-wer-braucht-leistung/</t>
+          <t>https://franksfinanzcheck.de/posts/hausratversicherung-wer-braucht-leistung/</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -3785,7 +3785,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/heizperiode-vorbereiten-spaetsommer/</t>
+          <t>https://franksfinanzcheck.de/posts/heizperiode-vorbereiten-spaetsommer/</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/kfz-versicherung-wechseln/</t>
+          <t>https://franksfinanzcheck.de/posts/kfz-versicherung-wechseln/</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -3829,7 +3829,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/kostenloses-girokonto-finden/</t>
+          <t>https://franksfinanzcheck.de/posts/kostenloses-girokonto-finden/</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/kreditkarte-ohne-jahresgebuehr/</t>
+          <t>https://franksfinanzcheck.de/posts/kreditkarte-ohne-jahresgebuehr/</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -3873,7 +3873,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/last-minute-urlaubsangebote-sichern/</t>
+          <t>https://franksfinanzcheck.de/posts/last-minute-urlaubsangebote-sichern/</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -3895,7 +3895,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-buchen-so-sparst-du/</t>
+          <t>https://franksfinanzcheck.de/posts/mietwagen-buchen-so-sparst-du/</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -3917,7 +3917,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/mietwagen-fallen-vermeiden/</t>
+          <t>https://franksfinanzcheck.de/posts/mietwagen-fallen-vermeiden/</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
+          <t>https://franksfinanzcheck.de/posts/notgroschen-aufbauen-wie-viel-reicht/</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -3961,7 +3961,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/private-unfallversicherung-fuer-wen-sie-sich-wirklich-lohnt/</t>
+          <t>https://franksfinanzcheck.de/posts/private-unfallversicherung-fuer-wen-sie-sich-wirklich-lohnt/</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/privathaftpflicht-warum-pflicht-kosten/</t>
+          <t>https://franksfinanzcheck.de/posts/privathaftpflicht-warum-pflicht-kosten/</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -4005,7 +4005,7 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/ratenkredit-bestszins-vergleichen/</t>
+          <t>https://franksfinanzcheck.de/posts/ratenkredit-bestszins-vergleichen/</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
@@ -4027,7 +4027,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/reisekrankenversicherung-wann-lohnt/</t>
+          <t>https://franksfinanzcheck.de/posts/reisekrankenversicherung-wann-lohnt/</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -4049,7 +4049,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/strom-sparen-haushalt-20-tipps/</t>
+          <t>https://franksfinanzcheck.de/posts/strom-sparen-haushalt-20-tipps/</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
@@ -4071,7 +4071,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromanbieter-wechseln-2026/</t>
+          <t>https://franksfinanzcheck.de/posts/stromanbieter-wechseln-2026/</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/stromfresser-im-haushalt-entlarven/</t>
+          <t>https://franksfinanzcheck.de/posts/stromfresser-im-haushalt-entlarven/</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
@@ -4115,7 +4115,7 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/tagesgeld-zinsen-sicher-anlegen/</t>
+          <t>https://franksfinanzcheck.de/posts/tagesgeld-zinsen-sicher-anlegen/</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
@@ -4137,7 +4137,7 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/urlaubskasse-aufbessern-spartipps/</t>
+          <t>https://franksfinanzcheck.de/posts/urlaubskasse-aufbessern-spartipps/</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
@@ -4159,7 +4159,7 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/waermepumpe-vs-gasheizung-2026/</t>
+          <t>https://franksfinanzcheck.de/posts/waermepumpe-vs-gasheizung-2026/</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
@@ -4181,7 +4181,7 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/wlan-verstaerker-vs-mesh-wlan/</t>
+          <t>https://franksfinanzcheck.de/posts/wlan-verstaerker-vs-mesh-wlan/</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
@@ -4203,7 +4203,7 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>https://DEINE-DOMAIN.DE/posts/zahnzusatzversicherung-lohnt-sich/</t>
+          <t>https://franksfinanzcheck.de/posts/zahnzusatzversicherung-lohnt-sich/</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
@@ -4659,9 +4659,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
@@ -4704,9 +4702,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
@@ -4724,7 +4720,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   DEINE-DOMAIN.DE durch deine echte Domain ersetzen (hugo.toml baseURL).</t>
+          <t xml:space="preserve">   franksfinanzcheck.de durch deine echte Domain ersetzen (hugo.toml baseURL).</t>
         </is>
       </c>
     </row>
@@ -4763,9 +4759,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
@@ -4808,9 +4802,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>

</xml_diff>